<commit_message>
D2 + EC1 — retire instrument_type and element_class, add elementClass dictionary
D2: ri_properties.xml#instrument_type retired — the planned instrument's kind is now stated
via diggs-schema's new AbstractTargetObjectType/plannedEquipment, dictionary-checked against
the existing equipmentClass.xml without any change needed there.

EC1: new elementClass.xml codelist (trial/test/production/sacrificial), bound to both
diggs:RIColumn/elementClass and the new diggs:TargetRIColumn/elementClass. Retires
ri_properties.xml#element_class.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/ri_properties.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/ri_properties.xlsx
@@ -1010,7 +1010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="7" customWidth="1" style="2" min="1" max="1"/>
@@ -1068,58 +1068,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <f>IF(ISNA(VLOOKUP(B2,AssociatedElements!B$2:B2940,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B3,AssociatedElements!B$2:B2941,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>element_class</t>
+          <t>tested_fraction</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>Element class</t>
+          <t>Tested fraction of population</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>The role a planned or constructed rigid inclusion plays in the works, as distinct from what it is made of or how it is built. A trial element is installed before production to prove the method or calibrate the design and is normally not part of the permanent works; a test element is a production element selected for verification testing; a production element carries permanent load and is not tested destructively; a sacrificial element is installed to be tested to failure. The distinction governs which acceptance criteria apply and how a test result may be extrapolated, which is why it needs to be stated rather than inferred from whether a test happens to be attached.</t>
+          <t>The proportion of a planned population of elements that is to be tested, where a testing provision is scoped to a population rather than to named elements - "5 percent of production rigid inclusions". A FRACTION OF A POPULATION, NOT A RATE IN TIME: it answers "how many of them" and not "how often", and it is deliberately named to keep it distinct from the temporal reading frequency carried by diggs:TargetMeasurementType/readingFrequency. diggs:ProgramScopeType states WHICH features a provision governs, by geometry, layout or feature type, and has no fraction concept by design; this parameter states what share of that scoped population is sampled. The two are complementary and both are normally needed.</t>
         </is>
       </c>
       <c r="E2" s="13" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="n"/>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
       <c r="G2" s="9" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <f>IF(ISNA(VLOOKUP(B3,AssociatedElements!B$2:B2941,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>tested_fraction</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>Tested fraction of population</t>
-        </is>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>The proportion of a planned population of elements that is to be tested, where a testing provision is scoped to a population rather than to named elements - "5 percent of production rigid inclusions". A FRACTION OF A POPULATION, NOT A RATE IN TIME: it answers "how many of them" and not "how often", and it is deliberately named to keep it distinct from the temporal reading frequency carried by diggs:TargetMeasurementType/readingFrequency. diggs:ProgramScopeType states WHICH features a provision governs, by geometry, layout or feature type, and has no fraction concept by design; this parameter states what share of that scoped population is sampled. The two are complementary and both are normally needed.</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
+        <f>IF(ISNA(VLOOKUP(B4,AssociatedElements!B$2:B2942,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>test_load_pct_design_load</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Test load as percentage of design load</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The maximum load a planned load test is to reach, expressed as a percentage of the design working load of the element being tested. Stated as a ratio rather than as a force because the test requirement is written that way in practice and because the absolute value differs per element while the ratio does not, which is what lets one population-scoped test provision govern a whole zone. Where the provision is adopted from a standard or a published recommendation rather than derived for the project, carry it as a diggs:ProvenancedParameter and state that in the derivation property.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>double</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>dimensionless</t>
         </is>
@@ -1128,121 +1132,82 @@
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <f>IF(ISNA(VLOOKUP(B4,AssociatedElements!B$2:B2942,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B6,AssociatedElements!B$2:B2944,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>test_load_pct_design_load</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Test load as percentage of design load</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>The maximum load a planned load test is to reach, expressed as a percentage of the design working load of the element being tested. Stated as a ratio rather than as a force because the test requirement is written that way in practice and because the absolute value differs per element while the ratio does not, which is what lets one population-scoped test provision govern a whole zone. Where the provision is adopted from a standard or a published recommendation rather than derived for the project, carry it as a diggs:ProvenancedParameter and state that in the derivation property.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+          <t>testing_density</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Testing density</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>How densely a planned measurement is to be spaced across a population or an area, where the provision is a spatial or count-based density rather than a rate in time - one test per footing, one per linear foot of wall, one per unit area of slab (V2 Post-installation row 22: LTP special-inspection frequency/regime). DISTINCT FROM tested_fraction (what share of a population is tested) and from diggs:TargetMeasurementType/readingFrequency (a temporal rate): this states how closely spaced testing is in space or by count, which readingFrequency's reciprocal-time unit cannot express. The unit varies with what is being inspected - reciprocal length, reciprocal area, or a bare count per discrete element - so no single quantityClass is stated here; give the value with whatever unit fits the foundation type being described.</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>double</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>dimensionless</t>
         </is>
       </c>
       <c r="G4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <f>IF(ISNA(VLOOKUP(B5,AssociatedElements!B$2:B2943,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>instrument_type</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>Instrument type</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>The kind of instrument a planned monitoring measurement is to be taken with.
-THE PROPERTY IS DEFINED HERE; ITS VALUES COME FROM equipmentClass.xml. The two are not competing and neither is redundant. This entry declares that a planned measurement may state which instrument it is to be taken with, and that the value is a string; equipmentClass.xml declares what the permitted instrument names are. Take the value from https://diggsml.org/def/codes/DIGGS/0.1/equipmentClass.xml - piezometer, inclinometer, extensometer, earth_pressure_cell and the rest.
-Why the property stays here rather than moving wholesale. The vocabulary is entirely generic - a piezometer is a piezometer on any project - and it now lives in the generic codelist accordingly. But the PROPERTY is a parameter on a planned measurement, and there is no equipment reference on diggs:TargetMeasurementType for it to become instead: a plan cannot cite an Equipment feature that will not exist until the instrument is installed, and a plan-to-realized reference is forbidden outright. So the instrument kind is stated as a parameter, with its value governed by the equipment codelist. If a planned equipment object is ever added to the Target family, this entry becomes redundant and should be deprecated in favour of it.
-Superseded the earlier plan to promote this entry out of the RI dictionary (2026-08-16): promoting the VOCABULARY was right and has been done; promoting the property had nowhere to go.</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F5" s="13" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B7,AssociatedElements!B$2:B2945,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
       <c r="G5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <f>IF(ISNA(VLOOKUP(B6,AssociatedElements!B$2:B2944,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>testing_density</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Testing density</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>How densely a planned measurement is to be spaced across a population or an area, where the provision is a spatial or count-based density rather than a rate in time - one test per footing, one per linear foot of wall, one per unit area of slab (V2 Post-installation row 22: LTP special-inspection frequency/regime). DISTINCT FROM tested_fraction (what share of a population is tested) and from diggs:TargetMeasurementType/readingFrequency (a temporal rate): this states how closely spaced testing is in space or by count, which readingFrequency's reciprocal-time unit cannot express. The unit varies with what is being inspected - reciprocal length, reciprocal area, or a bare count per discrete element - so no single quantityClass is stated here; give the value with whatever unit fits the foundation type being described.</t>
-        </is>
-      </c>
-      <c r="E6" s="17" t="inlineStr">
-        <is>
-          <t>double</t>
-        </is>
+        <f>IF(ISNA(VLOOKUP(B8,AssociatedElements!B$2:B2946,1,FALSE)),"Not used","")</f>
+        <v/>
       </c>
       <c r="G6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <f>IF(ISNA(VLOOKUP(B7,AssociatedElements!B$2:B2945,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
+        <f>IF(ISNA(VLOOKUP(B9,AssociatedElements!B$2:B2947,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="17" t="n"/>
       <c r="G7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <f>IF(ISNA(VLOOKUP(B8,AssociatedElements!B$2:B2946,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
+        <f>IF(ISNA(VLOOKUP(B10,AssociatedElements!B$2:B2948,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B8" s="13" t="n"/>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="13" t="n"/>
+      <c r="F8" s="13" t="n"/>
       <c r="G8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <f>IF(ISNA(VLOOKUP(B9,AssociatedElements!B$2:B2947,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="16" t="n"/>
-      <c r="E9" s="17" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B11,AssociatedElements!B$2:B2949,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="14" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
       <c r="G9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <f>IF(ISNA(VLOOKUP(B10,AssociatedElements!B$2:B2948,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B12,AssociatedElements!B$2:B2950,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B10" s="13" t="n"/>
@@ -1254,7 +1219,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2">
-        <f>IF(ISNA(VLOOKUP(B11,AssociatedElements!B$2:B2949,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B13,AssociatedElements!B$2:B2951,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B11" s="13" t="n"/>
@@ -1266,7 +1231,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2">
-        <f>IF(ISNA(VLOOKUP(B12,AssociatedElements!B$2:B2950,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B14,AssociatedElements!B$2:B2952,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B12" s="13" t="n"/>
@@ -1278,31 +1243,31 @@
     </row>
     <row r="13">
       <c r="A13" s="2">
-        <f>IF(ISNA(VLOOKUP(B13,AssociatedElements!B$2:B2951,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B15,AssociatedElements!B$2:B2953,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B13" s="13" t="n"/>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="14" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
       <c r="G13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2">
-        <f>IF(ISNA(VLOOKUP(B14,AssociatedElements!B$2:B2952,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B16,AssociatedElements!B$2:B2954,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B14" s="13" t="n"/>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
+      <c r="C14" s="18" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="18" t="n"/>
+      <c r="F14" s="18" t="n"/>
       <c r="G14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2">
-        <f>IF(ISNA(VLOOKUP(B15,AssociatedElements!B$2:B2953,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B17,AssociatedElements!B$2:B2955,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B15" s="13" t="n"/>
@@ -1314,7 +1279,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2">
-        <f>IF(ISNA(VLOOKUP(B16,AssociatedElements!B$2:B2954,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B18,AssociatedElements!B$2:B2956,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B16" s="13" t="n"/>
@@ -1326,7 +1291,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2">
-        <f>IF(ISNA(VLOOKUP(B17,AssociatedElements!B$2:B2955,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B19,AssociatedElements!B$2:B2957,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B17" s="13" t="n"/>
@@ -1338,7 +1303,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2">
-        <f>IF(ISNA(VLOOKUP(B18,AssociatedElements!B$2:B2956,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B20,AssociatedElements!B$2:B2958,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B18" s="13" t="n"/>
@@ -1350,7 +1315,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2">
-        <f>IF(ISNA(VLOOKUP(B19,AssociatedElements!B$2:B2957,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B21,AssociatedElements!B$2:B2959,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B19" s="13" t="n"/>
@@ -1362,7 +1327,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2">
-        <f>IF(ISNA(VLOOKUP(B20,AssociatedElements!B$2:B2958,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B22,AssociatedElements!B$2:B2960,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B20" s="13" t="n"/>
@@ -1374,7 +1339,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2">
-        <f>IF(ISNA(VLOOKUP(B21,AssociatedElements!B$2:B2959,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B23,AssociatedElements!B$2:B2961,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B21" s="13" t="n"/>
@@ -1386,73 +1351,73 @@
     </row>
     <row r="22">
       <c r="A22" s="2">
-        <f>IF(ISNA(VLOOKUP(B22,AssociatedElements!B$2:B2960,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B24,AssociatedElements!B$2:B2962,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="D22" s="16" t="n"/>
       <c r="G22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2">
-        <f>IF(ISNA(VLOOKUP(B23,AssociatedElements!B$2:B2961,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B25,AssociatedElements!B$2:B2963,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B23" s="13" t="n"/>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="13" t="n"/>
       <c r="G23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2">
-        <f>IF(ISNA(VLOOKUP(B24,AssociatedElements!B$2:B2962,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="D24" s="16" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B26,AssociatedElements!B$2:B2964,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="13" t="n"/>
       <c r="G24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2">
-        <f>IF(ISNA(VLOOKUP(B25,AssociatedElements!B$2:B2963,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B27,AssociatedElements!B$2:B2965,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B25" s="13" t="n"/>
       <c r="C25" s="13" t="n"/>
+      <c r="D25" s="15" t="n"/>
       <c r="E25" s="13" t="n"/>
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2">
-        <f>IF(ISNA(VLOOKUP(B26,AssociatedElements!B$2:B2964,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B28,AssociatedElements!B$2:B2966,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B26" s="13" t="n"/>
       <c r="C26" s="13" t="n"/>
+      <c r="D26" s="14" t="n"/>
       <c r="E26" s="13" t="n"/>
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2">
-        <f>IF(ISNA(VLOOKUP(B27,AssociatedElements!B$2:B2965,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B29,AssociatedElements!B$2:B2967,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B27" s="13" t="n"/>
       <c r="C27" s="13" t="n"/>
-      <c r="D27" s="15" t="n"/>
+      <c r="D27" s="14" t="n"/>
       <c r="E27" s="13" t="n"/>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2">
-        <f>IF(ISNA(VLOOKUP(B28,AssociatedElements!B$2:B2966,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B30,AssociatedElements!B$2:B2968,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B28" s="13" t="n"/>
@@ -1464,31 +1429,31 @@
     </row>
     <row r="29">
       <c r="A29" s="2">
-        <f>IF(ISNA(VLOOKUP(B29,AssociatedElements!B$2:B2967,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B31,AssociatedElements!B$2:B2969,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B29" s="13" t="n"/>
-      <c r="C29" s="13" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13" t="n"/>
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="19" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="18" t="n"/>
       <c r="G29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2">
-        <f>IF(ISNA(VLOOKUP(B30,AssociatedElements!B$2:B2968,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B32,AssociatedElements!B$2:B2970,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B30" s="13" t="n"/>
-      <c r="C30" s="13" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
       <c r="G30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2">
-        <f>IF(ISNA(VLOOKUP(B31,AssociatedElements!B$2:B2969,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B33,AssociatedElements!B$2:B2971,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B31" s="13" t="n"/>
@@ -1500,7 +1465,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2">
-        <f>IF(ISNA(VLOOKUP(B32,AssociatedElements!B$2:B2970,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B34,AssociatedElements!B$2:B2972,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B32" s="13" t="n"/>
@@ -1512,7 +1477,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2">
-        <f>IF(ISNA(VLOOKUP(B33,AssociatedElements!B$2:B2971,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B35,AssociatedElements!B$2:B2973,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B33" s="13" t="n"/>
@@ -1524,7 +1489,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2">
-        <f>IF(ISNA(VLOOKUP(B34,AssociatedElements!B$2:B2972,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B36,AssociatedElements!B$2:B2974,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B34" s="13" t="n"/>
@@ -1536,34 +1501,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2">
-        <f>IF(ISNA(VLOOKUP(B35,AssociatedElements!B$2:B2973,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B35" s="13" t="n"/>
-      <c r="C35" s="18" t="n"/>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="18" t="n"/>
-      <c r="F35" s="18" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B37,AssociatedElements!B$2:B2975,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
       <c r="G35" s="9" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2">
-        <f>IF(ISNA(VLOOKUP(B36,AssociatedElements!B$2:B2974,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B36" s="13" t="n"/>
-      <c r="C36" s="18" t="n"/>
-      <c r="D36" s="19" t="n"/>
-      <c r="E36" s="18" t="n"/>
-      <c r="F36" s="18" t="n"/>
-      <c r="G36" s="9" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2">
-        <f>IF(ISNA(VLOOKUP(B37,AssociatedElements!B$2:B2975,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="G37" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1580,7 +1521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="6.83203125" customWidth="1" min="1" max="1"/>
@@ -1613,12 +1554,12 @@
     </row>
     <row r="2">
       <c r="A2">
-        <f>IF(ISNA(VLOOKUP(#REF!,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>element_class</t>
+        <f>IF(ISNA(VLOOKUP(B3,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t>tested_fraction</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1629,12 +1570,12 @@
     </row>
     <row r="3">
       <c r="A3">
-        <f>IF(ISNA(VLOOKUP(B3,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>tested_fraction</t>
+        <f>IF(ISNA(VLOOKUP(B4,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>test_load_pct_design_load</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1645,273 +1586,241 @@
     </row>
     <row r="4">
       <c r="A4">
-        <f>IF(ISNA(VLOOKUP(B4,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B6,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>test_load_pct_design_load</t>
+          <t>testing_density</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:testingDensity</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <f>IF(ISNA(VLOOKUP(B5,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>instrument_type</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>//diggs:parameterName</t>
-        </is>
-      </c>
+        <f>IF(ISNA(VLOOKUP(B7,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6">
-        <f>IF(ISNA(VLOOKUP(B6,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>testing_density</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>//diggs:parameterName</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>ancestor::diggs:testingDensity</t>
-        </is>
-      </c>
+        <f>IF(ISNA(VLOOKUP(B8,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7">
-        <f>IF(ISNA(VLOOKUP(B7,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B9,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8">
-        <f>IF(ISNA(VLOOKUP(B8,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B8" s="2" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B8" s="20" t="n"/>
     </row>
     <row r="9">
       <c r="A9">
-        <f>IF(ISNA(VLOOKUP(B9,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B9" s="2" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B11,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B9" s="20" t="n"/>
     </row>
     <row r="10">
       <c r="A10">
-        <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B12,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B10" s="20" t="n"/>
     </row>
     <row r="11">
       <c r="A11">
-        <f>IF(ISNA(VLOOKUP(B11,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B13,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B11" s="20" t="n"/>
     </row>
     <row r="12">
       <c r="A12">
-        <f>IF(ISNA(VLOOKUP(B12,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B14,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B12" s="20" t="n"/>
     </row>
     <row r="13">
       <c r="A13">
-        <f>IF(ISNA(VLOOKUP(B13,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B13" s="20" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B15,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14">
-        <f>IF(ISNA(VLOOKUP(B14,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B14" s="20" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B16,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15">
-        <f>IF(ISNA(VLOOKUP(B15,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B17,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16">
-        <f>IF(ISNA(VLOOKUP(B16,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B18,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17">
-        <f>IF(ISNA(VLOOKUP(B17,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B17" s="2" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B19,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B17" s="20" t="n"/>
     </row>
     <row r="18">
       <c r="A18">
-        <f>IF(ISNA(VLOOKUP(B18,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B18" s="2" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B20,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B18" s="20" t="n"/>
     </row>
     <row r="19">
       <c r="A19">
-        <f>IF(ISNA(VLOOKUP(B19,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B21,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B19" s="20" t="n"/>
     </row>
     <row r="20">
       <c r="A20">
-        <f>IF(ISNA(VLOOKUP(B20,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B22,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B20" s="20" t="n"/>
     </row>
     <row r="21">
       <c r="A21">
-        <f>IF(ISNA(VLOOKUP(B21,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B21" s="20" t="n"/>
     </row>
     <row r="22">
       <c r="A22">
-        <f>IF(ISNA(VLOOKUP(B22,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B22" s="20" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23">
-        <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B23" s="20" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B25,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24">
-        <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B26,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25">
-        <f>IF(ISNA(VLOOKUP(B25,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B25" s="2" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26">
-        <f>IF(ISNA(VLOOKUP(B26,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B26" s="2" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B28,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B26" s="13" t="n"/>
     </row>
     <row r="27">
       <c r="A27">
-        <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B29,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="A28">
-        <f>IF(ISNA(VLOOKUP(B28,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B30,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B28" s="13" t="n"/>
     </row>
     <row r="29">
       <c r="A29">
-        <f>IF(ISNA(VLOOKUP(B29,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B29" s="13" t="n"/>
     </row>
     <row r="30">
       <c r="A30">
-        <f>IF(ISNA(VLOOKUP(B30,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B32,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B30" s="13" t="n"/>
     </row>
     <row r="31">
       <c r="A31">
-        <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B33,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B31" s="13" t="n"/>
     </row>
     <row r="32">
       <c r="A32">
-        <f>IF(ISNA(VLOOKUP(B32,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B34,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B32" s="13" t="n"/>
     </row>
     <row r="33">
       <c r="A33">
-        <f>IF(ISNA(VLOOKUP(B33,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B35,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B33" s="13" t="n"/>
     </row>
     <row r="34">
       <c r="A34">
-        <f>IF(ISNA(VLOOKUP(B34,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B36,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B34" s="13" t="n"/>
     </row>
     <row r="35">
       <c r="A35">
-        <f>IF(ISNA(VLOOKUP(B35,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B35" s="13" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36">
-        <f>IF(ISNA(VLOOKUP(B36,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B36" s="13" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37">
         <f>IF(ISNA(VLOOKUP(B37,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B37" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>